<commit_message>
fix(intelligence): make mailbox source reference optional
</commit_message>
<xml_diff>
--- a/SmartWorkplaceIntelligence/config/templates/SmartWorkplaceIntelligence-MailboxMigrationExceptions.xlsx
+++ b/SmartWorkplaceIntelligence/config/templates/SmartWorkplaceIntelligence-MailboxMigrationExceptions.xlsx
@@ -169,8 +169,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="MailboxMigrationExceptions" displayName="MailboxMigrationExceptions" ref="A7:J8" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="10">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="MailboxMigrationExceptions" displayName="MailboxMigrationExceptions" ref="A7:I8" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="9">
     <x:tableColumn id="1" name="Primary SMTP Address"/>
     <x:tableColumn id="2" name="Retain On-premises"/>
     <x:tableColumn id="3" name="Reason"/>
@@ -180,7 +180,6 @@
     <x:tableColumn id="7" name="Exchange GUID"/>
     <x:tableColumn id="8" name="AD Object GUID"/>
     <x:tableColumn id="9" name="Display Name"/>
-    <x:tableColumn id="10" name="Source Reference"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -393,7 +392,6 @@
     <x:col min="7" max="7" width="39" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="39" hidden="0" customWidth="1"/>
     <x:col min="9" max="9" width="32" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="65" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="22" customHeight="1">
@@ -406,7 +404,6 @@
       <x:c r="G1" s="2"/>
       <x:c r="H1" s="2"/>
       <x:c r="I1" s="2"/>
-      <x:c r="J1" s="2"/>
     </x:row>
     <x:row r="2" ht="30" customHeight="1">
       <x:c r="A2" s="3" t="str">
@@ -420,7 +417,6 @@
       <x:c r="G2" s="2"/>
       <x:c r="H2" s="2"/>
       <x:c r="I2" s="2"/>
-      <x:c r="J2" s="2"/>
     </x:row>
     <x:row r="3" ht="22" customHeight="1">
       <x:c r="A3" s="2"/>
@@ -432,7 +428,6 @@
       <x:c r="G3" s="2"/>
       <x:c r="H3" s="2"/>
       <x:c r="I3" s="2"/>
-      <x:c r="J3" s="2"/>
     </x:row>
     <x:row r="4" ht="22" customHeight="1">
       <x:c r="A4" s="2" t="str">
@@ -454,7 +449,6 @@
       <x:c r="G4" s="2"/>
       <x:c r="H4" s="2"/>
       <x:c r="I4" s="2"/>
-      <x:c r="J4" s="2"/>
     </x:row>
     <x:row r="5" ht="22" customHeight="1">
       <x:c r="A5" s="6" t="str">
@@ -468,7 +462,6 @@
       <x:c r="G5" s="2"/>
       <x:c r="H5" s="2"/>
       <x:c r="I5" s="2"/>
-      <x:c r="J5" s="2"/>
     </x:row>
     <x:row r="6" ht="22" customHeight="1">
       <x:c r="A6" s="2"/>
@@ -480,7 +473,6 @@
       <x:c r="G6" s="2"/>
       <x:c r="H6" s="2"/>
       <x:c r="I6" s="2"/>
-      <x:c r="J6" s="2"/>
     </x:row>
     <x:row r="7" ht="34" customHeight="1">
       <x:c r="A7" s="10" t="str">
@@ -510,9 +502,6 @@
       <x:c r="I7" s="10" t="str">
         <x:v>Display Name</x:v>
       </x:c>
-      <x:c r="J7" s="10" t="str">
-        <x:v>Source Reference</x:v>
-      </x:c>
     </x:row>
     <x:row r="8" ht="22" customHeight="1">
       <x:c r="A8" s="11"/>
@@ -524,7 +513,6 @@
       <x:c r="G8" s="16"/>
       <x:c r="H8" s="16"/>
       <x:c r="I8" s="12"/>
-      <x:c r="J8" s="12"/>
     </x:row>
     <x:row r="9">
       <x:c r="E9" s="15"/>
@@ -30672,14 +30660,7 @@
         <x:v>Optional display label. It is never used to match a mailbox.</x:v>
       </x:c>
     </x:row>
-    <x:row r="17" ht="40" customHeight="1">
-      <x:c r="A17" s="19" t="str">
-        <x:v>Source Reference</x:v>
-      </x:c>
-      <x:c r="B17" s="18" t="str">
-        <x:v>Imported rows retain their original workbook, sheet and row reference. New manual rows can leave this blank.</x:v>
-      </x:c>
-    </x:row>
+    <x:row r="17" ht="40" customHeight="1"/>
     <x:row r="18" ht="40" customHeight="1">
       <x:c r="A18" s="19" t="str">
         <x:v>Counts above the table</x:v>

</xml_diff>

<commit_message>
docs(intelligence): update mailbox exception template guide
</commit_message>
<xml_diff>
--- a/SmartWorkplaceIntelligence/config/templates/SmartWorkplaceIntelligence-MailboxMigrationExceptions.xlsx
+++ b/SmartWorkplaceIntelligence/config/templates/SmartWorkplaceIntelligence-MailboxMigrationExceptions.xlsx
@@ -30592,16 +30592,20 @@
       <x:c r="A8" s="19" t="str">
         <x:v>Entry table</x:v>
       </x:c>
-      <x:c r="B8" s="18" t="str">
-        <x:v>Edit the Exceptions sheet. Keep the MailboxMigrationExceptions table and its column headers. Add rows inside the table.</x:v>
+      <x:c r="B8" s="18" t="inlineStr">
+        <x:is>
+          <x:t>Edit the nine-column MailboxMigrationExceptions table on Exceptions. Keep the headers and their order; add records inside the table. Source Reference is not part of this workbook.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="9" ht="40" customHeight="1">
       <x:c r="A9" s="19" t="str">
         <x:v>Primary SMTP Address</x:v>
       </x:c>
-      <x:c r="B9" s="18" t="str">
-        <x:v>Required for address-only entries. Enter one exact primary SMTP address per row. No wildcards, lists or display-name matching.</x:v>
+      <x:c r="B9" s="18" t="inlineStr">
+        <x:is>
+          <x:t>Enter one exact primary SMTP address per row. SMTP-only matches require reviewed identity confirmation. No wildcards, lists, aliases or display-name matching.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="10" ht="40" customHeight="1">
@@ -30616,8 +30620,10 @@
       <x:c r="A11" s="19" t="str">
         <x:v>Reason</x:v>
       </x:c>
-      <x:c r="B11" s="18" t="str">
-        <x:v>Recommended. Record the business or technical reason. Missing imported comments remain blank and are flagged for documentation review.</x:v>
+      <x:c r="B11" s="18" t="inlineStr">
+        <x:is>
+          <x:t>Record the current business or technical reason. A missing reason is a documentation warning; it does not cancel a valid, confirmed Yes decision.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="12" ht="40" customHeight="1">
@@ -30632,8 +30638,10 @@
       <x:c r="A13" s="19" t="str">
         <x:v>Decision Date</x:v>
       </x:c>
-      <x:c r="B13" s="18" t="str">
-        <x:v>Optional. Enter the actual decision date as an Excel date. Do not use the import date as the decision date.</x:v>
+      <x:c r="B13" s="18" t="inlineStr">
+        <x:is>
+          <x:t>Enter the actual decision date as an Excel date or ISO yyyy-mm-dd text. Do not substitute the import date.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="14" ht="40" customHeight="1">
@@ -30648,8 +30656,10 @@
       <x:c r="A15" s="19" t="str">
         <x:v>Technical identity</x:v>
       </x:c>
-      <x:c r="B15" s="18" t="str">
-        <x:v>Exchange GUID and AD Object GUID are reserved for reviewed inventory binding. Do not guess them. This draft has no protected cells or automatic lookup.</x:v>
+      <x:c r="B15" s="18" t="inlineStr">
+        <x:is>
+          <x:t>Enter only reviewed Exchange GUID and AD Object GUID values from the matching inventory identity. Never guess. Unknown or conflicting GUIDs require review; there is no automatic lookup or write-back.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="16" ht="40" customHeight="1">
@@ -30665,24 +30675,30 @@
       <x:c r="A18" s="19" t="str">
         <x:v>Counts above the table</x:v>
       </x:c>
-      <x:c r="B18" s="18" t="str">
-        <x:v>Listed addresses and Marked Yes are input-row counts, not qualified distinct mailbox counts.</x:v>
+      <x:c r="B18" s="18" t="inlineStr">
+        <x:is>
+          <x:t>Listed addresses and Marked Yes count input rows in rows 8-5007, not qualified distinct mailboxes. Beyond 5,000 rows, extend the counters and dropdowns; preparation reads the actual table range.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="19" ht="40" customHeight="1">
       <x:c r="A19" s="19" t="str">
         <x:v>Matching</x:v>
       </x:c>
-      <x:c r="B19" s="18" t="str">
-        <x:v>The future preparation step will resolve one mailbox identity and check that it is still local. Unmatched or ambiguous rows require review.</x:v>
+      <x:c r="B19" s="18" t="inlineStr">
+        <x:is>
+          <x:t>Preparation resolves confirmed technical identities or approved private bindings against qualified inventories. A unique SMTP-only match still requires binding confirmation; unresolved or conflicting identities require review.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="20" ht="40" customHeight="1">
       <x:c r="A20" s="19" t="str">
         <x:v>Power BI count</x:v>
       </x:c>
-      <x:c r="B20" s="18" t="str">
-        <x:v>Only distinct, active, uniquely matched local mailboxes can contribute to the retained count. Missing source or unqualified coverage is Not measured, not zero.</x:v>
+      <x:c r="B20" s="18" t="inlineStr">
+        <x:is>
+          <x:t>Power BI displays counts from the validated preparation snapshot. Only unique, conflict-free local planning identities marked Yes count as retained. Missing or unqualified evidence is not a verified zero.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="21" ht="40" customHeight="1">
@@ -30697,8 +30713,10 @@
       <x:c r="A22" s="19" t="str">
         <x:v>Updates</x:v>
       </x:c>
-      <x:c r="B22" s="18" t="str">
-        <x:v>Save the shared workbook. Changes appear after the next validated preparation and a report refresh. Upload and integration are separate deployment steps.</x:v>
+      <x:c r="B22" s="18" t="inlineStr">
+        <x:is>
+          <x:t>Save the shared workbook. Changes appear only after validated preparation, transfer of the resulting batch where required, and report refresh. Saving this file does not run those steps.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="23" ht="40" customHeight="1">

</xml_diff>